<commit_message>
Elimino "Historic" del PiGs a GestioProducte
</commit_message>
<xml_diff>
--- a/Docs/Diferencies entre PiGs Meus i Self.xlsx
+++ b/Docs/Diferencies entre PiGs Meus i Self.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\_Actiu\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71836F31-A402-4074-BC26-05E3D274F1E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B198EF06-C5FD-42D9-861E-0244AC932116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{6BF5068B-93F7-4D64-8F2C-C2F86CB2EFAE}"/>
+    <workbookView xWindow="19090" yWindow="-20" windowWidth="19420" windowHeight="10420" xr2:uid="{6BF5068B-93F7-4D64-8F2C-C2F86CB2EFAE}"/>
   </bookViews>
   <sheets>
     <sheet name="PiGs 12-12-2022" sheetId="3" r:id="rId1"/>
@@ -21,14 +21,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -505,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF8A5D0D-B8B5-43EE-9A3C-77A80F538C29}">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
@@ -514,7 +506,7 @@
     <col min="8" max="8" width="1.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="5">
         <v>44907</v>
       </c>
@@ -537,7 +529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -562,7 +554,7 @@
         <v>-9.9999999999909051E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -587,7 +579,7 @@
         <v>5.4199999999999591</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -612,7 +604,7 @@
         <v>-1085.1199999999953</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -637,7 +629,7 @@
         <v>1.0200000000004366</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -662,7 +654,7 @@
         <v>-0.1300000000000523</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -687,7 +679,7 @@
         <v>-1.9099999999998545</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>0</v>
       </c>
@@ -716,14 +708,14 @@
         <v>-1080.7300000000105</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>21</v>
       </c>
@@ -734,12 +726,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="J13" s="1">
+        <v>1160.78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>10</v>
       </c>
@@ -750,7 +745,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>16</v>
       </c>
@@ -762,7 +757,7 @@
         <v>366.05200000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>15</v>
       </c>

</xml_diff>